<commit_message>
Save project code and data
</commit_message>
<xml_diff>
--- a/Structure_Data/test/20260703_02/structure_factor_20260703_02.xlsx
+++ b/Structure_Data/test/20260703_02/structure_factor_20260703_02.xlsx
@@ -40,7 +40,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:C33"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -248,6 +248,153 @@
         <v>10.4494593749493</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">瓶颈度 beta / Constrictivity (x)</t>
+        </is>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">瓶颈半径 r_min (um)</t>
+        </is>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">孔体半径 r_max (um)</t>
+        </is>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">瓶颈度状态 / Constrictivity Status</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Radius (um)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CPSD (total volume fraction)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIP (total volume fraction)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>0</v>
+      </c>
+      <c r="B26">
+        <v>0.568698883056641</v>
+      </c>
+      <c r="C26">
+        <v>0.566329956054688</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>0.5</v>
+      </c>
+      <c r="B27">
+        <v>0.568698883056641</v>
+      </c>
+      <c r="C27">
+        <v>0.566329956054688</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>1</v>
+      </c>
+      <c r="B28">
+        <v>0.381446838378906</v>
+      </c>
+      <c r="C28">
+        <v>0.32977294921875</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>1.5</v>
+      </c>
+      <c r="B29">
+        <v>0.180255889892578</v>
+      </c>
+      <c r="C29">
+        <v>0.0242996215820312</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>2</v>
+      </c>
+      <c r="B30">
+        <v>0.0547370910644531</v>
+      </c>
+      <c r="C30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>2.5</v>
+      </c>
+      <c r="B31">
+        <v>0.009613037109375</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>3</v>
+      </c>
+      <c r="B32">
+        <v>0</v>
+      </c>
+      <c r="C32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>3.5</v>
+      </c>
+      <c r="B33">
+        <v>0</v>
+      </c>
+      <c r="C33">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>